<commit_message>
Add vivid day 1 post designs, launch Reel, approved pricing and WhatsApp details
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0199j6yvtjnLVs9SvDCZskf8
</commit_message>
<xml_diff>
--- a/projects/pro-core-media/content/ProCoreMedia-Content-Dashboard.xlsx
+++ b/projects/pro-core-media/content/ProCoreMedia-Content-Dashboard.xlsx
@@ -643,7 +643,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -696,7 +696,7 @@
           <t>مرحبًا بكم في ProCore Media 🖤 وكالة إعلانات وتسويق رقمي سعودية، نجمع بين الإبداع والذكاء الاصطناعي والبيانات لنصنع لعلامتك حضورًا يليق بها ونتائج تُقاس.
 تابعونا… القادم أجمل.
 👉 تابعنا وأرسل لنا رسالة
-📩 راسلنا على واتساب: [رابط واتساب]</t>
+📩 واتساب: 0594943048 — https://wa.me/966594943048</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
@@ -765,7 +765,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
@@ -829,7 +829,7 @@
 4) تصميم الهوية البصرية
 أي خدمة تحتاجها أولًا؟ اكتبها في التعليقات 👇
 👉 اكتب (خدمات) في الرسائل
-📩 راسلنا على واتساب: [رابط واتساب]</t>
+📩 واتساب: 0594943048 — https://wa.me/966594943048</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
@@ -898,7 +898,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -949,7 +949,7 @@
         <is>
           <t>هكذا تبدأ القصة ✨ ProCore Media… حيث يلتقي الإبداع بالابتكار.
 👉 تابع الحساب
-📩 راسلنا على واتساب: [رابط واتساب]</t>
+📩 واتساب: 0594943048 — https://wa.me/966594943048</t>
         </is>
       </c>
       <c r="N4" s="2" t="inlineStr">
@@ -1018,7 +1018,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -1077,7 +1077,7 @@
 3) تنفيذ وتقرير شهري واضح
 احجز استشارتك الآن 📩
 👉 احجز استشارة عبر واتساب
-📩 راسلنا على واتساب: [رابط واتساب]</t>
+📩 واتساب: 0594943048 — https://wa.me/966594943048</t>
         </is>
       </c>
       <c r="N5" s="2" t="inlineStr">
@@ -1146,7 +1146,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -1199,7 +1199,7 @@
           <t>هل تنشر باستمرار والتفاعل ضعيف؟ غالبًا السبب واحد من هذه الأخطاء الخمسة 👇
 احفظ المنشور وراجع حسابك عليها.
 👉 احفظ المنشور + شاركه
-📩 راسلنا على واتساب: [رابط واتساب]</t>
+📩 واتساب: 0594943048 — https://wa.me/966594943048</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
@@ -1268,7 +1268,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
@@ -1321,7 +1321,7 @@
           <t>خلّ حساباتك تشتغل وأنت مركّز على نشاطك 💼
 في خدمة إدارة السوشيال نجهّز لك: خطة شهرية، تصاميم احترافية، نشر منتظم، متابعة التعليقات والرسائل، وتقرير أداء.
 👉 اسأل عن الباقات
-📩 راسلنا على واتساب: [رابط واتساب]</t>
+📩 واتساب: 0594943048 — https://wa.me/966594943048</t>
         </is>
       </c>
       <c r="N7" s="2" t="inlineStr">
@@ -1390,7 +1390,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -1443,7 +1443,7 @@
           <t>نفس المنتج… نتيجة مختلفة تمامًا 🤯 صورة عادية بالجوال تتحول لإعلان احترافي بمساعدة الذكاء الاصطناعي.
 (عينة توضيحية من إنتاجنا بالذكاء الاصطناعي — ليست لعميل)
 👉 تبي نجرّب على منتجك؟ راسلنا
-📩 راسلنا على واتساب: [رابط واتساب]</t>
+📩 واتساب: 0594943048 — https://wa.me/966594943048</t>
         </is>
       </c>
       <c r="N8" s="2" t="inlineStr">
@@ -1512,7 +1512,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
@@ -1563,7 +1563,7 @@
         <is>
           <t>سؤالنا الليلة 👇 اختر حرفًا واحدًا في التعليقات، وبنجاوب على أكثر تحدٍّ تكرر في منشور قادم.
 👉 علّق بحرف
-📩 راسلنا على واتساب: [رابط واتساب]</t>
+📩 واتساب: 0594943048 — https://wa.me/966594943048</t>
         </is>
       </c>
       <c r="N9" s="2" t="inlineStr">
@@ -1632,7 +1632,7 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -1687,7 +1687,7 @@
 Impressions = عدد مرات الظهور (الشخص الواحد قد يشاهده أكثر من مرة).
 لماذا يهمك الفرق؟ لأنه يكشف هل تصل لجمهور جديد أم تكرر الظهور لنفس الأشخاص.
 👉 احفظ المنشور
-📩 راسلنا على واتساب: [رابط واتساب]</t>
+📩 واتساب: 0594943048 — https://wa.me/966594943048</t>
         </is>
       </c>
       <c r="N10" s="2" t="inlineStr">
@@ -1756,7 +1756,7 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
@@ -1807,7 +1807,7 @@
         <is>
           <t>الإعلان الناجح ليس صدفة 🎯 نبني حملاتك على Facebook وInstagram خطوة بخطوة: جمهور واضح، إعلانات مصممة للتحويل، متابعة يومية، وتقرير يوضح أين صُرفت كل ريال.
 👉 اطلب خطة إعلانية
-📩 راسلنا على واتساب: [رابط واتساب]</t>
+📩 واتساب: 0594943048 — https://wa.me/966594943048</t>
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr">
@@ -1876,7 +1876,7 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
@@ -1927,7 +1927,7 @@
         <is>
           <t>الذكاء الاصطناعي ما يلغي الإبداع… يسرّعه ⚡ نستخدمه في: 1) توليد أفكار أكثر 2) إنتاج صور إعلانية 3) مشاهد فيديو — والقرار النهائي دائمًا لفريقنا.
 👉 تابعنا لمزيد من نصائح AI
-📩 راسلنا على واتساب: [رابط واتساب]</t>
+📩 واتساب: 0594943048 — https://wa.me/966594943048</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr">
@@ -1996,7 +1996,7 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
@@ -2047,7 +2047,7 @@
         <is>
           <t>مشروع تصوري (Concept) ☕ تخيّلنا حملة افتتاح لمقهى مختص في الخبر: فكرة، تصاميم، ورسالة واحدة واضحة. هذا نموذج إبداعي يوضح أسلوبنا — وليس عملًا لعميل.
 👉 تبي حملة لنشاطك؟ راسلنا
-📩 راسلنا على واتساب: [رابط واتساب]</t>
+📩 واتساب: 0594943048 — https://wa.me/966594943048</t>
         </is>
       </c>
       <c r="N13" s="2" t="inlineStr">
@@ -2116,7 +2116,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
@@ -2167,7 +2167,7 @@
         <is>
           <t>ما في وقت سحري يناسب الجميع ⏰ ابدأ بتجربة أوقات مختلفة لمدة أسبوعين، ثم افتح Insights وشوف متى جمهورك متصل أكثر. نحن نعتمد هذا الأسلوب مع كل حساب.
 👉 جرّبها وأخبرنا
-📩 راسلنا على واتساب: [رابط واتساب]</t>
+📩 واتساب: 0594943048 — https://wa.me/966594943048</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr">
@@ -2236,7 +2236,7 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
@@ -2287,7 +2287,7 @@
         <is>
           <t>الفيديو القصير هو أقوى أداة وصول اليوم 🎬 ننتج لك Reels من الفكرة إلى المونتاج — بالتصوير أو بمشاهد مولّدة بالذكاء الاصطناعي.
 👉 اطلب فكرة Reel لنشاطك
-📩 راسلنا على واتساب: [رابط واتساب]</t>
+📩 واتساب: 0594943048 — https://wa.me/966594943048</t>
         </is>
       </c>
       <c r="N15" s="2" t="inlineStr">
@@ -2356,7 +2356,7 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
@@ -2408,7 +2408,7 @@
           <t>مشهد سينمائي أُنتج بالكامل بالذكاء الاصطناعي 🍽️ هذا النوع من المشاهد يمكن استخدامه في إعلانات المطاعم بتكلفة أقل من التصوير التقليدي.
 (عينة توضيحية — ليست لعميل)
 👉 تبي مشهد لنشاطك؟ راسلنا
-📩 راسلنا على واتساب: [رابط واتساب]</t>
+📩 واتساب: 0594943048 — https://wa.me/966594943048</t>
         </is>
       </c>
       <c r="N16" s="2" t="inlineStr">
@@ -2477,7 +2477,7 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
@@ -2527,7 +2527,7 @@
         <is>
           <t>تصميمان لنفس الإعلان… أيهما يجذبك أكثر؟ 👀 علّق بـ A أو B — وبنكشف بكرة ليش الفرق مهم في الإعلانات.
 👉 علّق A أو B
-📩 راسلنا على واتساب: [رابط واتساب]</t>
+📩 واتساب: 0594943048 — https://wa.me/966594943048</t>
         </is>
       </c>
       <c r="N17" s="2" t="inlineStr">
@@ -2596,7 +2596,7 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
@@ -2647,7 +2647,7 @@
         <is>
           <t>أول سطر في منشورك هو الإعلان الحقيقي ✍️ 5 صيغ تساعدك: سؤال مباشر، رقم مفاجئ، خطأ شائع، وعد واضح، قصة قصيرة. أي صيغة تستخدمها أكثر؟
 👉 احفظ + جرّب
-📩 راسلنا على واتساب: [رابط واتساب]</t>
+📩 واتساب: 0594943048 — https://wa.me/966594943048</t>
         </is>
       </c>
       <c r="N18" s="2" t="inlineStr">
@@ -2716,7 +2716,7 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
@@ -2767,7 +2767,7 @@
         <is>
           <t>قبل ما يقرأ العميل كلمة واحدة، هويتك تكون تكلمت عنك 🎨 نصمم لك شعارًا ونظام ألوان وخطوط وتطبيقات جاهزة للسوشيال والمطبوعات.
 👉 اطلب عرض هوية
-📩 راسلنا على واتساب: [رابط واتساب]</t>
+📩 واتساب: 0594943048 — https://wa.me/966594943048</t>
         </is>
       </c>
       <c r="N19" s="2" t="inlineStr">
@@ -2836,7 +2836,7 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
@@ -2886,7 +2886,7 @@
         <is>
           <t>من فكرة على ورقة إلى منشور جاهز 🛠️ هكذا نشتغل: بحث، فكرة، تصميم، مراجعة، ثم نشر في الوقت المناسب.
 👉 تابعنا
-📩 راسلنا على واتساب: [رابط واتساب]</t>
+📩 واتساب: 0594943048 — https://wa.me/966594943048</t>
         </is>
       </c>
       <c r="N20" s="2" t="inlineStr">
@@ -2955,7 +2955,7 @@
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
@@ -2980,12 +2980,12 @@
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>Image ⚠️</t>
+          <t>Image</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>عرض: مراجعة مجانية لحسابك (يحتاج موافقة)</t>
+          <t>عرض: مراجعة مجانية لحسابك (معتمد)</t>
         </is>
       </c>
       <c r="K21" s="2" t="inlineStr">
@@ -3006,7 +3006,7 @@
         <is>
           <t>نقدم مراجعة مجانية لحسابات نشاطك على Instagram وFacebook مع 3 توصيات عملية تقدر تطبقها فورًا ✅ العرض لأول 10 منشآت.
 👉 أرسل رابط حسابك على واتساب
-📩 راسلنا على واتساب: [رابط واتساب]</t>
+📩 واتساب: 0594943048 — https://wa.me/966594943048</t>
         </is>
       </c>
       <c r="N21" s="2" t="inlineStr">
@@ -3042,7 +3042,7 @@
       </c>
       <c r="U21" s="2" t="inlineStr">
         <is>
-          <t>Pending approval — needs offer/pricing approval</t>
+          <t>Pending approval</t>
         </is>
       </c>
       <c r="V21" s="2" t="inlineStr">
@@ -3075,7 +3075,7 @@
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
@@ -3125,7 +3125,7 @@
         <is>
           <t>3 مبادئ لا نتنازل عنها: وضوح في الخطة، إبداع في التنفيذ، وأرقام تُقاس في النهاية 🖤
 👉 تابعنا
-📩 راسلنا على واتساب: [رابط واتساب]</t>
+📩 واتساب: 0594943048 — https://wa.me/966594943048</t>
         </is>
       </c>
       <c r="N22" s="2" t="inlineStr">
@@ -3194,7 +3194,7 @@
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
@@ -3245,7 +3245,7 @@
         <is>
           <t>مشروع تصوري (Concept) 🏡 إعلان لمشروع فلل فاخر بأسلوب الهوية الذهبية. نموذج يوضح أسلوبنا في التسويق العقاري — وليس عملًا لعميل.
 👉 عندك مشروع عقاري؟ راسلنا
-📩 راسلنا على واتساب: [رابط واتساب]</t>
+📩 واتساب: 0594943048 — https://wa.me/966594943048</t>
         </is>
       </c>
       <c r="N23" s="2" t="inlineStr">
@@ -3314,7 +3314,7 @@
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
@@ -3365,7 +3365,7 @@
         <is>
           <t>كيف تتغير صورة النشاط لما تتطور هويته ✨ (مشروع تصوري للتوضيح — ليس لعميل)
 👉 اطلب عرض هوية
-📩 راسلنا على واتساب: [رابط واتساب]</t>
+📩 واتساب: 0594943048 — https://wa.me/966594943048</t>
         </is>
       </c>
       <c r="N24" s="2" t="inlineStr">
@@ -3434,7 +3434,7 @@
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
@@ -3485,7 +3485,7 @@
         <is>
           <t>تحدٍّ اليوم 💡 اكتب نوع نشاطك في التعليقات (مطعم، عيادة، عقار، متجر…) وفريقنا يقترح عليك فكرة منشور مجانًا.
 👉 علّق بنوع نشاطك
-📩 راسلنا على واتساب: [رابط واتساب]</t>
+📩 واتساب: 0594943048 — https://wa.me/966594943048</t>
         </is>
       </c>
       <c r="N25" s="2" t="inlineStr">
@@ -3554,7 +3554,7 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-17</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
@@ -3605,7 +3605,7 @@
         <is>
           <t>سؤال نسمعه كثيرًا 💰 ابدأ بميزانية اختبار صغيرة، جرّب أكثر من إعلان، ثم ضاعف الصرف على الأفضل أداءً. القرار يكون بالأرقام لا بالتخمين.
 👉 احفظ المنشور
-📩 راسلنا على واتساب: [رابط واتساب]</t>
+📩 واتساب: 0594943048 — https://wa.me/966594943048</t>
         </is>
       </c>
       <c r="N26" s="2" t="inlineStr">
@@ -3674,7 +3674,7 @@
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-17</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
@@ -3699,12 +3699,12 @@
       </c>
       <c r="I27" s="2" t="inlineStr">
         <is>
-          <t>Image ⚠️</t>
+          <t>Image</t>
         </is>
       </c>
       <c r="J27" s="2" t="inlineStr">
         <is>
-          <t>باقاتنا: Start · Growth · Pro (بعد اعتماد الأسعار)</t>
+          <t>باقاتنا: Start · Growth · Pro (تبدأ من 1,875 ر.س)</t>
         </is>
       </c>
       <c r="K27" s="2" t="inlineStr">
@@ -3725,7 +3725,7 @@
         <is>
           <t>سواء كنت تبدأ أو تبي تكبر بسرعة، عندنا باقة تناسبك 📦 اطلب تفاصيل الباقات وقارن بنفسك.
 👉 اطلب الباقات
-📩 راسلنا على واتساب: [رابط واتساب]</t>
+📩 واتساب: 0594943048 — https://wa.me/966594943048</t>
         </is>
       </c>
       <c r="N27" s="2" t="inlineStr">
@@ -3761,7 +3761,7 @@
       </c>
       <c r="U27" s="2" t="inlineStr">
         <is>
-          <t>Pending approval — needs offer/pricing approval</t>
+          <t>Pending approval</t>
         </is>
       </c>
       <c r="V27" s="2" t="inlineStr">
@@ -3794,7 +3794,7 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-17</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
@@ -3846,7 +3846,7 @@
           <t>تخيّلنا إعلانًا لأكاديمية سباحة للأطفال 🏊 مشاهد مولّدة بالذكاء الاصطناعي توضح كيف يمكن عرض تجربة الأطفال بشكل جذاب.
 (نموذج تصوري — ليس لعميل)
 👉 عندك أكاديمية أو نادٍ؟ راسلنا
-📩 راسلنا على واتساب: [رابط واتساب]</t>
+📩 واتساب: 0594943048 — https://wa.me/966594943048</t>
         </is>
       </c>
       <c r="N28" s="2" t="inlineStr">
@@ -3915,7 +3915,7 @@
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-17</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
@@ -3966,7 +3966,7 @@
         <is>
           <t>أسبوع أول مليء بالأفكار 🙌 شكرًا لكل من تابعنا وتفاعل. إذا تبي نخطط محتوى وإعلانات نشاطك للشهر القادم، احجز استشارتك الآن.
 👉 احجز استشارة
-📩 راسلنا على واتساب: [رابط واتساب]</t>
+📩 واتساب: 0594943048 — https://wa.me/966594943048</t>
         </is>
       </c>
       <c r="N29" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Record day 1 Metricool drafts and statuses in the content dashboard
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0199j6yvtjnLVs9SvDCZskf8
</commit_message>
<xml_diff>
--- a/projects/pro-core-media/content/ProCoreMedia-Content-Dashboard.xlsx
+++ b/projects/pro-core-media/content/ProCoreMedia-Content-Dashboard.xlsx
@@ -724,10 +724,14 @@
           <t>1080×1350</t>
         </is>
       </c>
-      <c r="S2" s="2" t="inlineStr"/>
+      <c r="S2" s="2" t="inlineStr">
+        <is>
+          <t>design/agency/out/posts-v2/D1-P1-launch.jpg</t>
+        </is>
+      </c>
       <c r="T2" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Ready</t>
         </is>
       </c>
       <c r="U2" s="2" t="inlineStr">
@@ -737,7 +741,7 @@
       </c>
       <c r="V2" s="2" t="inlineStr">
         <is>
-          <t>Not scheduled</t>
+          <t>Draft in Metricool (IG 392974341, FB 392974471)</t>
         </is>
       </c>
       <c r="W2" s="2" t="inlineStr"/>
@@ -749,7 +753,11 @@
       <c r="AC2" s="2" t="inlineStr"/>
       <c r="AD2" s="2" t="inlineStr"/>
       <c r="AE2" s="2" t="inlineStr"/>
-      <c r="AF2" s="2" t="inlineStr"/>
+      <c r="AF2" s="2" t="inlineStr">
+        <is>
+          <t>Vivid v2 design</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -857,10 +865,14 @@
           <t>1080×1350 ×5</t>
         </is>
       </c>
-      <c r="S3" s="2" t="inlineStr"/>
+      <c r="S3" s="2" t="inlineStr">
+        <is>
+          <t>design/agency/out/posts-v2/D1-P2-01..05-*.jpg</t>
+        </is>
+      </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Ready</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
@@ -870,7 +882,7 @@
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>Not scheduled</t>
+          <t>Draft in Metricool (IG 392974682, FB 392974923)</t>
         </is>
       </c>
       <c r="W3" s="2" t="inlineStr"/>
@@ -882,7 +894,11 @@
       <c r="AC3" s="2" t="inlineStr"/>
       <c r="AD3" s="2" t="inlineStr"/>
       <c r="AE3" s="2" t="inlineStr"/>
-      <c r="AF3" s="2" t="inlineStr"/>
+      <c r="AF3" s="2" t="inlineStr">
+        <is>
+          <t>Carousel 5 slides</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -977,10 +993,14 @@
           <t>1080×1920</t>
         </is>
       </c>
-      <c r="S4" s="2" t="inlineStr"/>
+      <c r="S4" s="2" t="inlineStr">
+        <is>
+          <t>design/agency/out/posts-v2/D1-P3-launch-reel.mp4</t>
+        </is>
+      </c>
       <c r="T4" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Ready</t>
         </is>
       </c>
       <c r="U4" s="2" t="inlineStr">
@@ -990,7 +1010,7 @@
       </c>
       <c r="V4" s="2" t="inlineStr">
         <is>
-          <t>Not scheduled</t>
+          <t>Draft in Metricool (IG 392975000, FB 392975044)</t>
         </is>
       </c>
       <c r="W4" s="2" t="inlineStr"/>
@@ -1002,7 +1022,11 @@
       <c r="AC4" s="2" t="inlineStr"/>
       <c r="AD4" s="2" t="inlineStr"/>
       <c r="AE4" s="2" t="inlineStr"/>
-      <c r="AF4" s="2" t="inlineStr"/>
+      <c r="AF4" s="2" t="inlineStr">
+        <is>
+          <t>12s Reel, silent — add audio in-app if desired</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -1105,10 +1129,14 @@
           <t>1080×1350</t>
         </is>
       </c>
-      <c r="S5" s="2" t="inlineStr"/>
+      <c r="S5" s="2" t="inlineStr">
+        <is>
+          <t>design/agency/out/posts-v2/D1-P4-how-we-start.jpg</t>
+        </is>
+      </c>
       <c r="T5" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Ready</t>
         </is>
       </c>
       <c r="U5" s="2" t="inlineStr">
@@ -1118,7 +1146,7 @@
       </c>
       <c r="V5" s="2" t="inlineStr">
         <is>
-          <t>Not scheduled</t>
+          <t>Draft in Metricool (IG 392975084, FB 392975122)</t>
         </is>
       </c>
       <c r="W5" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
Schedule day 1 posts in Metricool and record statuses
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0199j6yvtjnLVs9SvDCZskf8
</commit_message>
<xml_diff>
--- a/projects/pro-core-media/content/ProCoreMedia-Content-Dashboard.xlsx
+++ b/projects/pro-core-media/content/ProCoreMedia-Content-Dashboard.xlsx
@@ -726,7 +726,7 @@
       </c>
       <c r="S2" s="2" t="inlineStr">
         <is>
-          <t>design/agency/out/posts-v2/D1-P1-launch.jpg</t>
+          <t>design/agency/out/posts-v3/D1-P1-launch.jpg</t>
         </is>
       </c>
       <c r="T2" s="2" t="inlineStr">
@@ -736,12 +736,12 @@
       </c>
       <c r="U2" s="2" t="inlineStr">
         <is>
-          <t>Pending approval</t>
+          <t>Approved 2026-10-11</t>
         </is>
       </c>
       <c r="V2" s="2" t="inlineStr">
         <is>
-          <t>Draft in Metricool (IG 392974341, FB 392974471)</t>
+          <t>Scheduled 2026-10-11 09:00 (IG 392979440, FB 392979494)</t>
         </is>
       </c>
       <c r="W2" s="2" t="inlineStr"/>
@@ -755,7 +755,7 @@
       <c r="AE2" s="2" t="inlineStr"/>
       <c r="AF2" s="2" t="inlineStr">
         <is>
-          <t>Vivid v2 design</t>
+          <t>v3: AI photo + Saudi dialect; IG AI label on</t>
         </is>
       </c>
     </row>
@@ -867,7 +867,7 @@
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>design/agency/out/posts-v2/D1-P2-01..05-*.jpg</t>
+          <t>design/agency/out/posts-v3/D1-P2-01..05-*.jpg</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
@@ -877,12 +877,12 @@
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>Pending approval</t>
+          <t>Approved 2026-10-11</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>Draft in Metricool (IG 392974682, FB 392974923)</t>
+          <t>Scheduled 2026-10-11 13:30 (IG 392979514, FB 392979528)</t>
         </is>
       </c>
       <c r="W3" s="2" t="inlineStr"/>
@@ -896,7 +896,7 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>Carousel 5 slides</t>
+          <t>v3 carousel 5 slides; IG AI label on</t>
         </is>
       </c>
     </row>
@@ -1005,12 +1005,12 @@
       </c>
       <c r="U4" s="2" t="inlineStr">
         <is>
-          <t>Pending approval</t>
+          <t>Approved 2026-10-11</t>
         </is>
       </c>
       <c r="V4" s="2" t="inlineStr">
         <is>
-          <t>Draft in Metricool (IG 392975000, FB 392975044)</t>
+          <t>Scheduled 2026-10-11 17:30 (IG 392979544, FB 392979556)</t>
         </is>
       </c>
       <c r="W4" s="2" t="inlineStr"/>
@@ -1024,7 +1024,7 @@
       <c r="AE4" s="2" t="inlineStr"/>
       <c r="AF4" s="2" t="inlineStr">
         <is>
-          <t>12s Reel, silent — add audio in-app if desired</t>
+          <t>12s motion Reel, silent</t>
         </is>
       </c>
     </row>
@@ -1131,7 +1131,7 @@
       </c>
       <c r="S5" s="2" t="inlineStr">
         <is>
-          <t>design/agency/out/posts-v2/D1-P4-how-we-start.jpg</t>
+          <t>design/agency/out/posts-v3/D1-P4-how-we-start.jpg</t>
         </is>
       </c>
       <c r="T5" s="2" t="inlineStr">
@@ -1141,12 +1141,12 @@
       </c>
       <c r="U5" s="2" t="inlineStr">
         <is>
-          <t>Pending approval</t>
+          <t>Approved 2026-10-11</t>
         </is>
       </c>
       <c r="V5" s="2" t="inlineStr">
         <is>
-          <t>Draft in Metricool (IG 392975084, FB 392975122)</t>
+          <t>Scheduled 2026-10-11 21:00 (IG 392979577, FB 392979603)</t>
         </is>
       </c>
       <c r="W5" s="2" t="inlineStr"/>
@@ -1158,7 +1158,11 @@
       <c r="AC5" s="2" t="inlineStr"/>
       <c r="AD5" s="2" t="inlineStr"/>
       <c r="AE5" s="2" t="inlineStr"/>
-      <c r="AF5" s="2" t="inlineStr"/>
+      <c r="AF5" s="2" t="inlineStr">
+        <is>
+          <t>v3 + launch offer; IG AI label on</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">

</xml_diff>